<commit_message>
Bug fixes and improvements
</commit_message>
<xml_diff>
--- a/WebRoot/oem/cnpc/locale/locale-en.xlsx
+++ b/WebRoot/oem/cnpc/locale/locale-en.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A347DA5-4C62-4F4A-8648-572D52BB0E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7F4825-22EF-475C-B0A3-07B243A978C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="732" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="732" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6005" uniqueCount="4619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6313" uniqueCount="4850">
   <si>
     <t>myself</t>
   </si>
@@ -17167,6 +17167,776 @@
   <si>
     <t>interlock protection</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyUpscalingPparameters</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>升频参数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyUpscalingFullnessCoefficientLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>升频充满系数临界值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyUpperLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>频率上限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyUpscalingStepSize</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>升频步长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyUpscalingStabilityDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>单次升频稳定时长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyReductionParameters</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>降频参数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyReductionFullnessCoefficientLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>降频充满系数临界值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyLowerLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>频率下限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyReductionStepSize</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>降频步长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frequencyReductionStabilityDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>单次降频稳定时长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FSDiagramWorkTypeEnable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>工况使能</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-使能</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Up_FullnessCoefficientLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升频参数-升频充满系数临界值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Up_FrequencyUpperLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升频参数-频率上限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Up_StepSize</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升频参数-升频步长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Up_StabilityDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升频参数-单次升频稳定时长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Down_FullnessCoefficientLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-降频参数-降频充满系数临界值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Down_FrequencyLowerLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-降频参数-频率下限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Down_StepSize</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-降频参数-降频步长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversion_Down_StabilityDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-降频参数-单次降频稳定时长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1201</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-抽喷</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1202</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-正常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1203</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-充满不足</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1204</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-供液不足</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1205</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-供液极差</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1206</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-抽空</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1207</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-泵下堵</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1208</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-气锁</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1209</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-气影响</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1210</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-间隙漏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1212</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-游动凡尔漏失</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1213</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-固定凡尔漏失</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1214</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-双凡尔漏失</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1215</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-游动凡尔失灵/油管漏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1216</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-固定凡尔失灵</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1217</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-双凡尔失灵</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1218</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-上死点别碰</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1219</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-碰泵</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1220</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-活塞/底部断脱/未入工作筒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1221</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-柱塞脱出工作筒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1222</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-杆断脱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1223</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-杆泵卡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1224</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-结蜡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1225</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-严重结蜡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1226</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-出砂</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1227</t>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-严重出砂</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1230</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-惯性载荷大</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_FrequencyConversionEnable_FSDiagramWorkType1232</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能变频-升降频工况使能状态-采集异常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>联锁保护-使能</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1201</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-抽喷</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1202</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-正常</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1203</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-充满不足</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1204</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-供液不足</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1205</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-供液极差</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1206</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-抽空</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1207</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-泵下堵</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1208</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-气锁</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1209</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-气影响</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1210</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-间隙漏</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1212</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-游动凡尔漏失</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1213</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-固定凡尔漏失</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1214</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-双凡尔漏失</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1215</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-游动凡尔失灵/油管漏</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1216</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-固定凡尔失灵</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1217</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-双凡尔失灵</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1218</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-上死点别碰</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1219</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-碰泵</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1220</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-活塞/底部断脱/未入工作筒</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1221</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-柱塞脱出工作筒</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1222</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-杆断脱</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1223</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-杆泵卡</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1224</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-结蜡</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1225</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-严重结蜡</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1226</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-出砂</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1227</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-严重出砂</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1230</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-惯性载荷大</t>
+  </si>
+  <si>
+    <t>write_InterlockProtectionEnable_FSDiagramWorkType1232</t>
+  </si>
+  <si>
+    <t>联锁保护-工况使能状态-采集异常</t>
+  </si>
+  <si>
+    <t>Upscaling parameters</t>
+  </si>
+  <si>
+    <t>The critical value of the upscaling filling coefficient</t>
+  </si>
+  <si>
+    <t>Frequency cap</t>
+  </si>
+  <si>
+    <t>Upgrade step length</t>
+  </si>
+  <si>
+    <t>Stable duration of a single upscaling</t>
+  </si>
+  <si>
+    <t>Downclocking parameters</t>
+  </si>
+  <si>
+    <t>Downfill the coefficient threshold</t>
+  </si>
+  <si>
+    <t>Lower frequency limit</t>
+  </si>
+  <si>
+    <t>Frequency reduction step length</t>
+  </si>
+  <si>
+    <t>Stable duration of a single downturn</t>
+  </si>
+  <si>
+    <t>The working conditions are enabled</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - enable</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - boost parameter - boost fill factor critical value</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - upscaling parameters - frequency ceiling</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - upscaling parameters - upscaling step</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - upscaling parameters - stable duration of a single upscaling</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency reduction parameter - frequency reduction filling factor critical value</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency reduction parameter - lower frequency limit</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency reduction parameters - frequency reduction steps</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency reduction parameters - stable duration of a single frequency reduction</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working condition enabling state - pumping</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - normal</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - full of deficiencies</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working conditions enable state - insufficient liquid supply</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working conditions enable state - extremely poor liquid supply</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - evacuation</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - pump plugging</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working conditions enable state - air lock</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working conditions enable state-gas influence</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - gap leakage</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - swimming Vera leakage</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - fixed Vere leakage</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - double Vert leakage</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - swimming Verde failure/oil pipe leakage</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - fixed Verde failure</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state-double Versaille failure</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - do not touch the dead point</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working condition enabling state - touch pump</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working conditions enable state - piston/bottom disconnection/not entering the barrel</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - Enabling state of rising and falling frequency working conditions - plunger out of the working barrel</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - rod disconnection</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency lifting and reciprocating working conditions enable state - rod pump card</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working condition enabling state - waxing</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - enabling state under frequency up and down working conditions - severe waxing</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working conditions enable state - sand output</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - serious sand production</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency rise and fall working conditions enable state-inertia load is large</t>
+  </si>
+  <si>
+    <t>Intelligent frequency conversion - frequency up and down working conditions enable state - collect abnormal conditions</t>
+  </si>
+  <si>
+    <t>Interlock Protection - Enable</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - pumping spray</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - normal</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabled state - full of deficiencies</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - insufficient liquid supply</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - extremely poor liquid supply</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - evacuation</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - pump plugging</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - air lock</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - pneumatic influence</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - gap leakage</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - swimmer Ver leakage</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - fixed Vere leakage</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - double Verde leakage</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - swimming Verde failure/oil pipe leakage</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - fixed Verde failure</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - double Verde failure</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - do not touch the dead point</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - touch pump</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - piston / bottom disconnection/not entering the barrel</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - plunger out of the barrel</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - rod disconnection</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - rod pump card</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - waxing</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - severe waxing</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - sand discharge</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - serious sand discharge</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - large inertia load</t>
+  </si>
+  <si>
+    <t>Interlock protection - working condition enabling state - collection of abnormal conditions</t>
   </si>
 </sst>
 </file>
@@ -20550,7 +21320,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E372"/>
+  <dimension ref="A1:E449"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="38"/>
@@ -26883,6 +27653,1315 @@
       </c>
       <c r="E372" s="24" t="s">
         <v>4585</v>
+      </c>
+    </row>
+    <row r="373" spans="1:5">
+      <c r="A373" s="11">
+        <v>372</v>
+      </c>
+      <c r="B373" s="1" t="s">
+        <v>4619</v>
+      </c>
+      <c r="C373" s="7" t="s">
+        <v>4620</v>
+      </c>
+      <c r="D373" s="20" t="s">
+        <v>4773</v>
+      </c>
+      <c r="E373" s="24" t="s">
+        <v>4773</v>
+      </c>
+    </row>
+    <row r="374" spans="1:5">
+      <c r="A374" s="11">
+        <v>373</v>
+      </c>
+      <c r="B374" s="1" t="s">
+        <v>4621</v>
+      </c>
+      <c r="C374" s="7" t="s">
+        <v>4622</v>
+      </c>
+      <c r="D374" s="20" t="s">
+        <v>4774</v>
+      </c>
+      <c r="E374" s="24" t="s">
+        <v>4774</v>
+      </c>
+    </row>
+    <row r="375" spans="1:5">
+      <c r="A375" s="11">
+        <v>374</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>4623</v>
+      </c>
+      <c r="C375" s="7" t="s">
+        <v>4624</v>
+      </c>
+      <c r="D375" s="20" t="s">
+        <v>4775</v>
+      </c>
+      <c r="E375" s="24" t="s">
+        <v>4775</v>
+      </c>
+    </row>
+    <row r="376" spans="1:5">
+      <c r="A376" s="11">
+        <v>375</v>
+      </c>
+      <c r="B376" s="1" t="s">
+        <v>4625</v>
+      </c>
+      <c r="C376" s="7" t="s">
+        <v>4626</v>
+      </c>
+      <c r="D376" s="20" t="s">
+        <v>4776</v>
+      </c>
+      <c r="E376" s="24" t="s">
+        <v>4776</v>
+      </c>
+    </row>
+    <row r="377" spans="1:5">
+      <c r="A377" s="11">
+        <v>376</v>
+      </c>
+      <c r="B377" s="1" t="s">
+        <v>4627</v>
+      </c>
+      <c r="C377" s="7" t="s">
+        <v>4628</v>
+      </c>
+      <c r="D377" s="20" t="s">
+        <v>4777</v>
+      </c>
+      <c r="E377" s="24" t="s">
+        <v>4777</v>
+      </c>
+    </row>
+    <row r="378" spans="1:5">
+      <c r="A378" s="11">
+        <v>377</v>
+      </c>
+      <c r="B378" s="1" t="s">
+        <v>4629</v>
+      </c>
+      <c r="C378" s="7" t="s">
+        <v>4630</v>
+      </c>
+      <c r="D378" s="20" t="s">
+        <v>4778</v>
+      </c>
+      <c r="E378" s="24" t="s">
+        <v>4778</v>
+      </c>
+    </row>
+    <row r="379" spans="1:5">
+      <c r="A379" s="11">
+        <v>378</v>
+      </c>
+      <c r="B379" s="1" t="s">
+        <v>4631</v>
+      </c>
+      <c r="C379" s="7" t="s">
+        <v>4632</v>
+      </c>
+      <c r="D379" s="20" t="s">
+        <v>4779</v>
+      </c>
+      <c r="E379" s="24" t="s">
+        <v>4779</v>
+      </c>
+    </row>
+    <row r="380" spans="1:5">
+      <c r="A380" s="11">
+        <v>379</v>
+      </c>
+      <c r="B380" s="1" t="s">
+        <v>4633</v>
+      </c>
+      <c r="C380" s="7" t="s">
+        <v>4634</v>
+      </c>
+      <c r="D380" s="20" t="s">
+        <v>4780</v>
+      </c>
+      <c r="E380" s="24" t="s">
+        <v>4780</v>
+      </c>
+    </row>
+    <row r="381" spans="1:5">
+      <c r="A381" s="11">
+        <v>380</v>
+      </c>
+      <c r="B381" s="1" t="s">
+        <v>4635</v>
+      </c>
+      <c r="C381" s="7" t="s">
+        <v>4636</v>
+      </c>
+      <c r="D381" s="20" t="s">
+        <v>4781</v>
+      </c>
+      <c r="E381" s="24" t="s">
+        <v>4781</v>
+      </c>
+    </row>
+    <row r="382" spans="1:5">
+      <c r="A382" s="11">
+        <v>381</v>
+      </c>
+      <c r="B382" s="1" t="s">
+        <v>4637</v>
+      </c>
+      <c r="C382" s="7" t="s">
+        <v>4638</v>
+      </c>
+      <c r="D382" s="20" t="s">
+        <v>4782</v>
+      </c>
+      <c r="E382" s="24" t="s">
+        <v>4782</v>
+      </c>
+    </row>
+    <row r="383" spans="1:5">
+      <c r="A383" s="11">
+        <v>382</v>
+      </c>
+      <c r="B383" s="1" t="s">
+        <v>4639</v>
+      </c>
+      <c r="C383" s="7" t="s">
+        <v>4640</v>
+      </c>
+      <c r="D383" s="20" t="s">
+        <v>4783</v>
+      </c>
+      <c r="E383" s="24" t="s">
+        <v>4783</v>
+      </c>
+    </row>
+    <row r="384" spans="1:5">
+      <c r="A384" s="11">
+        <v>383</v>
+      </c>
+      <c r="B384" s="1" t="s">
+        <v>4641</v>
+      </c>
+      <c r="C384" s="7" t="s">
+        <v>4642</v>
+      </c>
+      <c r="D384" s="20" t="s">
+        <v>4784</v>
+      </c>
+      <c r="E384" s="24" t="s">
+        <v>4784</v>
+      </c>
+    </row>
+    <row r="385" spans="1:5">
+      <c r="A385" s="11">
+        <v>384</v>
+      </c>
+      <c r="B385" s="1" t="s">
+        <v>4643</v>
+      </c>
+      <c r="C385" s="7" t="s">
+        <v>4644</v>
+      </c>
+      <c r="D385" s="20" t="s">
+        <v>4785</v>
+      </c>
+      <c r="E385" s="24" t="s">
+        <v>4785</v>
+      </c>
+    </row>
+    <row r="386" spans="1:5">
+      <c r="A386" s="11">
+        <v>385</v>
+      </c>
+      <c r="B386" s="1" t="s">
+        <v>4645</v>
+      </c>
+      <c r="C386" s="7" t="s">
+        <v>4646</v>
+      </c>
+      <c r="D386" s="20" t="s">
+        <v>4786</v>
+      </c>
+      <c r="E386" s="24" t="s">
+        <v>4786</v>
+      </c>
+    </row>
+    <row r="387" spans="1:5">
+      <c r="A387" s="11">
+        <v>386</v>
+      </c>
+      <c r="B387" s="1" t="s">
+        <v>4647</v>
+      </c>
+      <c r="C387" s="7" t="s">
+        <v>4648</v>
+      </c>
+      <c r="D387" s="20" t="s">
+        <v>4787</v>
+      </c>
+      <c r="E387" s="24" t="s">
+        <v>4787</v>
+      </c>
+    </row>
+    <row r="388" spans="1:5">
+      <c r="A388" s="11">
+        <v>387</v>
+      </c>
+      <c r="B388" s="1" t="s">
+        <v>4649</v>
+      </c>
+      <c r="C388" s="7" t="s">
+        <v>4650</v>
+      </c>
+      <c r="D388" s="20" t="s">
+        <v>4788</v>
+      </c>
+      <c r="E388" s="24" t="s">
+        <v>4788</v>
+      </c>
+    </row>
+    <row r="389" spans="1:5">
+      <c r="A389" s="11">
+        <v>388</v>
+      </c>
+      <c r="B389" s="1" t="s">
+        <v>4651</v>
+      </c>
+      <c r="C389" s="7" t="s">
+        <v>4652</v>
+      </c>
+      <c r="D389" s="20" t="s">
+        <v>4789</v>
+      </c>
+      <c r="E389" s="24" t="s">
+        <v>4789</v>
+      </c>
+    </row>
+    <row r="390" spans="1:5">
+      <c r="A390" s="11">
+        <v>389</v>
+      </c>
+      <c r="B390" s="1" t="s">
+        <v>4653</v>
+      </c>
+      <c r="C390" s="7" t="s">
+        <v>4654</v>
+      </c>
+      <c r="D390" s="20" t="s">
+        <v>4790</v>
+      </c>
+      <c r="E390" s="24" t="s">
+        <v>4790</v>
+      </c>
+    </row>
+    <row r="391" spans="1:5">
+      <c r="A391" s="11">
+        <v>390</v>
+      </c>
+      <c r="B391" s="1" t="s">
+        <v>4655</v>
+      </c>
+      <c r="C391" s="7" t="s">
+        <v>4656</v>
+      </c>
+      <c r="D391" s="20" t="s">
+        <v>4791</v>
+      </c>
+      <c r="E391" s="24" t="s">
+        <v>4791</v>
+      </c>
+    </row>
+    <row r="392" spans="1:5">
+      <c r="A392" s="11">
+        <v>391</v>
+      </c>
+      <c r="B392" s="1" t="s">
+        <v>4657</v>
+      </c>
+      <c r="C392" s="7" t="s">
+        <v>4658</v>
+      </c>
+      <c r="D392" s="20" t="s">
+        <v>4792</v>
+      </c>
+      <c r="E392" s="24" t="s">
+        <v>4792</v>
+      </c>
+    </row>
+    <row r="393" spans="1:5">
+      <c r="A393" s="11">
+        <v>392</v>
+      </c>
+      <c r="B393" s="1" t="s">
+        <v>4659</v>
+      </c>
+      <c r="C393" s="7" t="s">
+        <v>4660</v>
+      </c>
+      <c r="D393" s="20" t="s">
+        <v>4793</v>
+      </c>
+      <c r="E393" s="24" t="s">
+        <v>4793</v>
+      </c>
+    </row>
+    <row r="394" spans="1:5">
+      <c r="A394" s="11">
+        <v>393</v>
+      </c>
+      <c r="B394" s="1" t="s">
+        <v>4661</v>
+      </c>
+      <c r="C394" s="7" t="s">
+        <v>4662</v>
+      </c>
+      <c r="D394" s="20" t="s">
+        <v>4794</v>
+      </c>
+      <c r="E394" s="24" t="s">
+        <v>4794</v>
+      </c>
+    </row>
+    <row r="395" spans="1:5">
+      <c r="A395" s="11">
+        <v>394</v>
+      </c>
+      <c r="B395" s="1" t="s">
+        <v>4663</v>
+      </c>
+      <c r="C395" s="7" t="s">
+        <v>4664</v>
+      </c>
+      <c r="D395" s="20" t="s">
+        <v>4795</v>
+      </c>
+      <c r="E395" s="24" t="s">
+        <v>4795</v>
+      </c>
+    </row>
+    <row r="396" spans="1:5">
+      <c r="A396" s="11">
+        <v>395</v>
+      </c>
+      <c r="B396" s="1" t="s">
+        <v>4665</v>
+      </c>
+      <c r="C396" s="7" t="s">
+        <v>4666</v>
+      </c>
+      <c r="D396" s="20" t="s">
+        <v>4796</v>
+      </c>
+      <c r="E396" s="24" t="s">
+        <v>4796</v>
+      </c>
+    </row>
+    <row r="397" spans="1:5">
+      <c r="A397" s="11">
+        <v>396</v>
+      </c>
+      <c r="B397" s="1" t="s">
+        <v>4667</v>
+      </c>
+      <c r="C397" s="7" t="s">
+        <v>4668</v>
+      </c>
+      <c r="D397" s="20" t="s">
+        <v>4797</v>
+      </c>
+      <c r="E397" s="24" t="s">
+        <v>4797</v>
+      </c>
+    </row>
+    <row r="398" spans="1:5">
+      <c r="A398" s="11">
+        <v>397</v>
+      </c>
+      <c r="B398" s="1" t="s">
+        <v>4669</v>
+      </c>
+      <c r="C398" s="7" t="s">
+        <v>4670</v>
+      </c>
+      <c r="D398" s="20" t="s">
+        <v>4798</v>
+      </c>
+      <c r="E398" s="24" t="s">
+        <v>4798</v>
+      </c>
+    </row>
+    <row r="399" spans="1:5">
+      <c r="A399" s="11">
+        <v>398</v>
+      </c>
+      <c r="B399" s="1" t="s">
+        <v>4671</v>
+      </c>
+      <c r="C399" s="7" t="s">
+        <v>4672</v>
+      </c>
+      <c r="D399" s="20" t="s">
+        <v>4799</v>
+      </c>
+      <c r="E399" s="24" t="s">
+        <v>4799</v>
+      </c>
+    </row>
+    <row r="400" spans="1:5">
+      <c r="A400" s="11">
+        <v>399</v>
+      </c>
+      <c r="B400" s="1" t="s">
+        <v>4673</v>
+      </c>
+      <c r="C400" s="7" t="s">
+        <v>4674</v>
+      </c>
+      <c r="D400" s="20" t="s">
+        <v>4800</v>
+      </c>
+      <c r="E400" s="24" t="s">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="401" spans="1:5">
+      <c r="A401" s="11">
+        <v>400</v>
+      </c>
+      <c r="B401" s="1" t="s">
+        <v>4675</v>
+      </c>
+      <c r="C401" s="7" t="s">
+        <v>4676</v>
+      </c>
+      <c r="D401" s="20" t="s">
+        <v>4801</v>
+      </c>
+      <c r="E401" s="24" t="s">
+        <v>4801</v>
+      </c>
+    </row>
+    <row r="402" spans="1:5">
+      <c r="A402" s="11">
+        <v>401</v>
+      </c>
+      <c r="B402" s="1" t="s">
+        <v>4677</v>
+      </c>
+      <c r="C402" s="7" t="s">
+        <v>4678</v>
+      </c>
+      <c r="D402" s="20" t="s">
+        <v>4802</v>
+      </c>
+      <c r="E402" s="24" t="s">
+        <v>4802</v>
+      </c>
+    </row>
+    <row r="403" spans="1:5">
+      <c r="A403" s="11">
+        <v>402</v>
+      </c>
+      <c r="B403" s="1" t="s">
+        <v>4679</v>
+      </c>
+      <c r="C403" s="7" t="s">
+        <v>4680</v>
+      </c>
+      <c r="D403" s="20" t="s">
+        <v>4803</v>
+      </c>
+      <c r="E403" s="24" t="s">
+        <v>4803</v>
+      </c>
+    </row>
+    <row r="404" spans="1:5">
+      <c r="A404" s="11">
+        <v>403</v>
+      </c>
+      <c r="B404" s="1" t="s">
+        <v>4681</v>
+      </c>
+      <c r="C404" s="7" t="s">
+        <v>4682</v>
+      </c>
+      <c r="D404" s="20" t="s">
+        <v>4804</v>
+      </c>
+      <c r="E404" s="24" t="s">
+        <v>4804</v>
+      </c>
+    </row>
+    <row r="405" spans="1:5">
+      <c r="A405" s="11">
+        <v>404</v>
+      </c>
+      <c r="B405" s="1" t="s">
+        <v>4683</v>
+      </c>
+      <c r="C405" s="7" t="s">
+        <v>4684</v>
+      </c>
+      <c r="D405" s="20" t="s">
+        <v>4805</v>
+      </c>
+      <c r="E405" s="24" t="s">
+        <v>4805</v>
+      </c>
+    </row>
+    <row r="406" spans="1:5">
+      <c r="A406" s="11">
+        <v>405</v>
+      </c>
+      <c r="B406" s="1" t="s">
+        <v>4685</v>
+      </c>
+      <c r="C406" s="7" t="s">
+        <v>4686</v>
+      </c>
+      <c r="D406" s="20" t="s">
+        <v>4806</v>
+      </c>
+      <c r="E406" s="24" t="s">
+        <v>4806</v>
+      </c>
+    </row>
+    <row r="407" spans="1:5">
+      <c r="A407" s="11">
+        <v>406</v>
+      </c>
+      <c r="B407" s="1" t="s">
+        <v>4687</v>
+      </c>
+      <c r="C407" s="7" t="s">
+        <v>4688</v>
+      </c>
+      <c r="D407" s="20" t="s">
+        <v>4807</v>
+      </c>
+      <c r="E407" s="24" t="s">
+        <v>4807</v>
+      </c>
+    </row>
+    <row r="408" spans="1:5">
+      <c r="A408" s="11">
+        <v>407</v>
+      </c>
+      <c r="B408" s="1" t="s">
+        <v>4689</v>
+      </c>
+      <c r="C408" s="7" t="s">
+        <v>4690</v>
+      </c>
+      <c r="D408" s="20" t="s">
+        <v>4808</v>
+      </c>
+      <c r="E408" s="24" t="s">
+        <v>4808</v>
+      </c>
+    </row>
+    <row r="409" spans="1:5">
+      <c r="A409" s="11">
+        <v>408</v>
+      </c>
+      <c r="B409" s="1" t="s">
+        <v>4691</v>
+      </c>
+      <c r="C409" s="7" t="s">
+        <v>4692</v>
+      </c>
+      <c r="D409" s="20" t="s">
+        <v>4809</v>
+      </c>
+      <c r="E409" s="24" t="s">
+        <v>4809</v>
+      </c>
+    </row>
+    <row r="410" spans="1:5">
+      <c r="A410" s="11">
+        <v>409</v>
+      </c>
+      <c r="B410" s="1" t="s">
+        <v>4693</v>
+      </c>
+      <c r="C410" s="7" t="s">
+        <v>4694</v>
+      </c>
+      <c r="D410" s="20" t="s">
+        <v>4810</v>
+      </c>
+      <c r="E410" s="24" t="s">
+        <v>4810</v>
+      </c>
+    </row>
+    <row r="411" spans="1:5">
+      <c r="A411" s="11">
+        <v>410</v>
+      </c>
+      <c r="B411" s="1" t="s">
+        <v>4695</v>
+      </c>
+      <c r="C411" s="7" t="s">
+        <v>4696</v>
+      </c>
+      <c r="D411" s="20" t="s">
+        <v>4811</v>
+      </c>
+      <c r="E411" s="24" t="s">
+        <v>4811</v>
+      </c>
+    </row>
+    <row r="412" spans="1:5">
+      <c r="A412" s="11">
+        <v>411</v>
+      </c>
+      <c r="B412" s="1" t="s">
+        <v>4697</v>
+      </c>
+      <c r="C412" s="7" t="s">
+        <v>4698</v>
+      </c>
+      <c r="D412" s="20" t="s">
+        <v>4812</v>
+      </c>
+      <c r="E412" s="24" t="s">
+        <v>4812</v>
+      </c>
+    </row>
+    <row r="413" spans="1:5">
+      <c r="A413" s="11">
+        <v>412</v>
+      </c>
+      <c r="B413" s="1" t="s">
+        <v>4699</v>
+      </c>
+      <c r="C413" s="7" t="s">
+        <v>4700</v>
+      </c>
+      <c r="D413" s="20" t="s">
+        <v>4813</v>
+      </c>
+      <c r="E413" s="24" t="s">
+        <v>4813</v>
+      </c>
+    </row>
+    <row r="414" spans="1:5">
+      <c r="A414" s="11">
+        <v>413</v>
+      </c>
+      <c r="B414" s="1" t="s">
+        <v>4701</v>
+      </c>
+      <c r="C414" s="7" t="s">
+        <v>4702</v>
+      </c>
+      <c r="D414" s="20" t="s">
+        <v>4814</v>
+      </c>
+      <c r="E414" s="24" t="s">
+        <v>4814</v>
+      </c>
+    </row>
+    <row r="415" spans="1:5">
+      <c r="A415" s="11">
+        <v>414</v>
+      </c>
+      <c r="B415" s="1" t="s">
+        <v>4703</v>
+      </c>
+      <c r="C415" s="7" t="s">
+        <v>4704</v>
+      </c>
+      <c r="D415" s="20" t="s">
+        <v>4815</v>
+      </c>
+      <c r="E415" s="24" t="s">
+        <v>4815</v>
+      </c>
+    </row>
+    <row r="416" spans="1:5">
+      <c r="A416" s="11">
+        <v>415</v>
+      </c>
+      <c r="B416" s="1" t="s">
+        <v>4705</v>
+      </c>
+      <c r="C416" s="7" t="s">
+        <v>4706</v>
+      </c>
+      <c r="D416" s="20" t="s">
+        <v>4816</v>
+      </c>
+      <c r="E416" s="24" t="s">
+        <v>4816</v>
+      </c>
+    </row>
+    <row r="417" spans="1:5">
+      <c r="A417" s="11">
+        <v>416</v>
+      </c>
+      <c r="B417" s="1" t="s">
+        <v>4707</v>
+      </c>
+      <c r="C417" s="7" t="s">
+        <v>4708</v>
+      </c>
+      <c r="D417" s="20" t="s">
+        <v>4817</v>
+      </c>
+      <c r="E417" s="24" t="s">
+        <v>4817</v>
+      </c>
+    </row>
+    <row r="418" spans="1:5">
+      <c r="A418" s="11">
+        <v>417</v>
+      </c>
+      <c r="B418" s="1" t="s">
+        <v>4709</v>
+      </c>
+      <c r="C418" s="7" t="s">
+        <v>4710</v>
+      </c>
+      <c r="D418" s="20" t="s">
+        <v>4818</v>
+      </c>
+      <c r="E418" s="24" t="s">
+        <v>4818</v>
+      </c>
+    </row>
+    <row r="419" spans="1:5">
+      <c r="A419" s="11">
+        <v>418</v>
+      </c>
+      <c r="B419" s="1" t="s">
+        <v>4711</v>
+      </c>
+      <c r="C419" s="7" t="s">
+        <v>4712</v>
+      </c>
+      <c r="D419" s="20" t="s">
+        <v>4819</v>
+      </c>
+      <c r="E419" s="24" t="s">
+        <v>4819</v>
+      </c>
+    </row>
+    <row r="420" spans="1:5">
+      <c r="A420" s="11">
+        <v>419</v>
+      </c>
+      <c r="B420" s="1" t="s">
+        <v>4713</v>
+      </c>
+      <c r="C420" s="7" t="s">
+        <v>4714</v>
+      </c>
+      <c r="D420" s="20" t="s">
+        <v>4820</v>
+      </c>
+      <c r="E420" s="24" t="s">
+        <v>4820</v>
+      </c>
+    </row>
+    <row r="421" spans="1:5">
+      <c r="A421" s="11">
+        <v>383</v>
+      </c>
+      <c r="B421" s="1" t="s">
+        <v>4715</v>
+      </c>
+      <c r="C421" s="7" t="s">
+        <v>4716</v>
+      </c>
+      <c r="D421" s="20" t="s">
+        <v>4821</v>
+      </c>
+      <c r="E421" s="24" t="s">
+        <v>4821</v>
+      </c>
+    </row>
+    <row r="422" spans="1:5">
+      <c r="A422" s="11">
+        <v>392</v>
+      </c>
+      <c r="B422" s="1" t="s">
+        <v>4717</v>
+      </c>
+      <c r="C422" s="7" t="s">
+        <v>4718</v>
+      </c>
+      <c r="D422" s="20" t="s">
+        <v>4822</v>
+      </c>
+      <c r="E422" s="24" t="s">
+        <v>4822</v>
+      </c>
+    </row>
+    <row r="423" spans="1:5">
+      <c r="A423" s="11">
+        <v>393</v>
+      </c>
+      <c r="B423" s="1" t="s">
+        <v>4719</v>
+      </c>
+      <c r="C423" s="7" t="s">
+        <v>4720</v>
+      </c>
+      <c r="D423" s="20" t="s">
+        <v>4823</v>
+      </c>
+      <c r="E423" s="24" t="s">
+        <v>4823</v>
+      </c>
+    </row>
+    <row r="424" spans="1:5">
+      <c r="A424" s="11">
+        <v>394</v>
+      </c>
+      <c r="B424" s="1" t="s">
+        <v>4721</v>
+      </c>
+      <c r="C424" s="7" t="s">
+        <v>4722</v>
+      </c>
+      <c r="D424" s="20" t="s">
+        <v>4824</v>
+      </c>
+      <c r="E424" s="24" t="s">
+        <v>4824</v>
+      </c>
+    </row>
+    <row r="425" spans="1:5">
+      <c r="A425" s="11">
+        <v>395</v>
+      </c>
+      <c r="B425" s="1" t="s">
+        <v>4723</v>
+      </c>
+      <c r="C425" s="7" t="s">
+        <v>4724</v>
+      </c>
+      <c r="D425" s="20" t="s">
+        <v>4825</v>
+      </c>
+      <c r="E425" s="24" t="s">
+        <v>4825</v>
+      </c>
+    </row>
+    <row r="426" spans="1:5">
+      <c r="A426" s="11">
+        <v>396</v>
+      </c>
+      <c r="B426" s="1" t="s">
+        <v>4725</v>
+      </c>
+      <c r="C426" s="7" t="s">
+        <v>4726</v>
+      </c>
+      <c r="D426" s="20" t="s">
+        <v>4826</v>
+      </c>
+      <c r="E426" s="24" t="s">
+        <v>4826</v>
+      </c>
+    </row>
+    <row r="427" spans="1:5">
+      <c r="A427" s="11">
+        <v>397</v>
+      </c>
+      <c r="B427" s="1" t="s">
+        <v>4727</v>
+      </c>
+      <c r="C427" s="7" t="s">
+        <v>4728</v>
+      </c>
+      <c r="D427" s="20" t="s">
+        <v>4827</v>
+      </c>
+      <c r="E427" s="24" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="428" spans="1:5">
+      <c r="A428" s="11">
+        <v>398</v>
+      </c>
+      <c r="B428" s="1" t="s">
+        <v>4729</v>
+      </c>
+      <c r="C428" s="7" t="s">
+        <v>4730</v>
+      </c>
+      <c r="D428" s="20" t="s">
+        <v>4828</v>
+      </c>
+      <c r="E428" s="24" t="s">
+        <v>4828</v>
+      </c>
+    </row>
+    <row r="429" spans="1:5">
+      <c r="A429" s="11">
+        <v>399</v>
+      </c>
+      <c r="B429" s="1" t="s">
+        <v>4731</v>
+      </c>
+      <c r="C429" s="7" t="s">
+        <v>4732</v>
+      </c>
+      <c r="D429" s="20" t="s">
+        <v>4829</v>
+      </c>
+      <c r="E429" s="24" t="s">
+        <v>4829</v>
+      </c>
+    </row>
+    <row r="430" spans="1:5">
+      <c r="A430" s="11">
+        <v>400</v>
+      </c>
+      <c r="B430" s="1" t="s">
+        <v>4733</v>
+      </c>
+      <c r="C430" s="7" t="s">
+        <v>4734</v>
+      </c>
+      <c r="D430" s="20" t="s">
+        <v>4830</v>
+      </c>
+      <c r="E430" s="24" t="s">
+        <v>4830</v>
+      </c>
+    </row>
+    <row r="431" spans="1:5">
+      <c r="A431" s="11">
+        <v>401</v>
+      </c>
+      <c r="B431" s="1" t="s">
+        <v>4735</v>
+      </c>
+      <c r="C431" s="7" t="s">
+        <v>4736</v>
+      </c>
+      <c r="D431" s="20" t="s">
+        <v>4831</v>
+      </c>
+      <c r="E431" s="24" t="s">
+        <v>4831</v>
+      </c>
+    </row>
+    <row r="432" spans="1:5">
+      <c r="A432" s="11">
+        <v>402</v>
+      </c>
+      <c r="B432" s="1" t="s">
+        <v>4737</v>
+      </c>
+      <c r="C432" s="7" t="s">
+        <v>4738</v>
+      </c>
+      <c r="D432" s="20" t="s">
+        <v>4832</v>
+      </c>
+      <c r="E432" s="24" t="s">
+        <v>4832</v>
+      </c>
+    </row>
+    <row r="433" spans="1:5">
+      <c r="A433" s="11">
+        <v>403</v>
+      </c>
+      <c r="B433" s="1" t="s">
+        <v>4739</v>
+      </c>
+      <c r="C433" s="7" t="s">
+        <v>4740</v>
+      </c>
+      <c r="D433" s="20" t="s">
+        <v>4833</v>
+      </c>
+      <c r="E433" s="24" t="s">
+        <v>4833</v>
+      </c>
+    </row>
+    <row r="434" spans="1:5">
+      <c r="A434" s="11">
+        <v>404</v>
+      </c>
+      <c r="B434" s="1" t="s">
+        <v>4741</v>
+      </c>
+      <c r="C434" s="7" t="s">
+        <v>4742</v>
+      </c>
+      <c r="D434" s="20" t="s">
+        <v>4834</v>
+      </c>
+      <c r="E434" s="24" t="s">
+        <v>4834</v>
+      </c>
+    </row>
+    <row r="435" spans="1:5">
+      <c r="A435" s="11">
+        <v>405</v>
+      </c>
+      <c r="B435" s="1" t="s">
+        <v>4743</v>
+      </c>
+      <c r="C435" s="7" t="s">
+        <v>4744</v>
+      </c>
+      <c r="D435" s="20" t="s">
+        <v>4835</v>
+      </c>
+      <c r="E435" s="24" t="s">
+        <v>4835</v>
+      </c>
+    </row>
+    <row r="436" spans="1:5">
+      <c r="A436" s="11">
+        <v>406</v>
+      </c>
+      <c r="B436" s="1" t="s">
+        <v>4745</v>
+      </c>
+      <c r="C436" s="7" t="s">
+        <v>4746</v>
+      </c>
+      <c r="D436" s="20" t="s">
+        <v>4836</v>
+      </c>
+      <c r="E436" s="24" t="s">
+        <v>4836</v>
+      </c>
+    </row>
+    <row r="437" spans="1:5">
+      <c r="A437" s="11">
+        <v>407</v>
+      </c>
+      <c r="B437" s="1" t="s">
+        <v>4747</v>
+      </c>
+      <c r="C437" s="7" t="s">
+        <v>4748</v>
+      </c>
+      <c r="D437" s="20" t="s">
+        <v>4837</v>
+      </c>
+      <c r="E437" s="24" t="s">
+        <v>4837</v>
+      </c>
+    </row>
+    <row r="438" spans="1:5">
+      <c r="A438" s="11">
+        <v>408</v>
+      </c>
+      <c r="B438" s="1" t="s">
+        <v>4749</v>
+      </c>
+      <c r="C438" s="7" t="s">
+        <v>4750</v>
+      </c>
+      <c r="D438" s="20" t="s">
+        <v>4838</v>
+      </c>
+      <c r="E438" s="24" t="s">
+        <v>4838</v>
+      </c>
+    </row>
+    <row r="439" spans="1:5">
+      <c r="A439" s="11">
+        <v>409</v>
+      </c>
+      <c r="B439" s="1" t="s">
+        <v>4751</v>
+      </c>
+      <c r="C439" s="7" t="s">
+        <v>4752</v>
+      </c>
+      <c r="D439" s="20" t="s">
+        <v>4839</v>
+      </c>
+      <c r="E439" s="24" t="s">
+        <v>4839</v>
+      </c>
+    </row>
+    <row r="440" spans="1:5">
+      <c r="A440" s="11">
+        <v>410</v>
+      </c>
+      <c r="B440" s="1" t="s">
+        <v>4753</v>
+      </c>
+      <c r="C440" s="7" t="s">
+        <v>4754</v>
+      </c>
+      <c r="D440" s="20" t="s">
+        <v>4840</v>
+      </c>
+      <c r="E440" s="24" t="s">
+        <v>4840</v>
+      </c>
+    </row>
+    <row r="441" spans="1:5">
+      <c r="A441" s="11">
+        <v>411</v>
+      </c>
+      <c r="B441" s="1" t="s">
+        <v>4755</v>
+      </c>
+      <c r="C441" s="7" t="s">
+        <v>4756</v>
+      </c>
+      <c r="D441" s="20" t="s">
+        <v>4841</v>
+      </c>
+      <c r="E441" s="24" t="s">
+        <v>4841</v>
+      </c>
+    </row>
+    <row r="442" spans="1:5">
+      <c r="A442" s="11">
+        <v>412</v>
+      </c>
+      <c r="B442" s="1" t="s">
+        <v>4757</v>
+      </c>
+      <c r="C442" s="7" t="s">
+        <v>4758</v>
+      </c>
+      <c r="D442" s="20" t="s">
+        <v>4842</v>
+      </c>
+      <c r="E442" s="24" t="s">
+        <v>4842</v>
+      </c>
+    </row>
+    <row r="443" spans="1:5">
+      <c r="A443" s="11">
+        <v>413</v>
+      </c>
+      <c r="B443" s="1" t="s">
+        <v>4759</v>
+      </c>
+      <c r="C443" s="7" t="s">
+        <v>4760</v>
+      </c>
+      <c r="D443" s="20" t="s">
+        <v>4843</v>
+      </c>
+      <c r="E443" s="24" t="s">
+        <v>4843</v>
+      </c>
+    </row>
+    <row r="444" spans="1:5">
+      <c r="A444" s="11">
+        <v>414</v>
+      </c>
+      <c r="B444" s="1" t="s">
+        <v>4761</v>
+      </c>
+      <c r="C444" s="7" t="s">
+        <v>4762</v>
+      </c>
+      <c r="D444" s="20" t="s">
+        <v>4844</v>
+      </c>
+      <c r="E444" s="24" t="s">
+        <v>4844</v>
+      </c>
+    </row>
+    <row r="445" spans="1:5">
+      <c r="A445" s="11">
+        <v>415</v>
+      </c>
+      <c r="B445" s="1" t="s">
+        <v>4763</v>
+      </c>
+      <c r="C445" s="7" t="s">
+        <v>4764</v>
+      </c>
+      <c r="D445" s="20" t="s">
+        <v>4845</v>
+      </c>
+      <c r="E445" s="24" t="s">
+        <v>4845</v>
+      </c>
+    </row>
+    <row r="446" spans="1:5">
+      <c r="A446" s="11">
+        <v>416</v>
+      </c>
+      <c r="B446" s="1" t="s">
+        <v>4765</v>
+      </c>
+      <c r="C446" s="7" t="s">
+        <v>4766</v>
+      </c>
+      <c r="D446" s="20" t="s">
+        <v>4846</v>
+      </c>
+      <c r="E446" s="24" t="s">
+        <v>4846</v>
+      </c>
+    </row>
+    <row r="447" spans="1:5">
+      <c r="A447" s="11">
+        <v>417</v>
+      </c>
+      <c r="B447" s="1" t="s">
+        <v>4767</v>
+      </c>
+      <c r="C447" s="7" t="s">
+        <v>4768</v>
+      </c>
+      <c r="D447" s="20" t="s">
+        <v>4847</v>
+      </c>
+      <c r="E447" s="24" t="s">
+        <v>4847</v>
+      </c>
+    </row>
+    <row r="448" spans="1:5">
+      <c r="A448" s="11">
+        <v>418</v>
+      </c>
+      <c r="B448" s="1" t="s">
+        <v>4769</v>
+      </c>
+      <c r="C448" s="7" t="s">
+        <v>4770</v>
+      </c>
+      <c r="D448" s="20" t="s">
+        <v>4848</v>
+      </c>
+      <c r="E448" s="24" t="s">
+        <v>4848</v>
+      </c>
+    </row>
+    <row r="449" spans="1:5">
+      <c r="A449" s="11">
+        <v>419</v>
+      </c>
+      <c r="B449" s="1" t="s">
+        <v>4771</v>
+      </c>
+      <c r="C449" s="7" t="s">
+        <v>4772</v>
+      </c>
+      <c r="D449" s="20" t="s">
+        <v>4849</v>
+      </c>
+      <c r="E449" s="24" t="s">
+        <v>4849</v>
       </c>
     </row>
   </sheetData>

</xml_diff>